<commit_message>
Refine frequency benchmark model
</commit_message>
<xml_diff>
--- a/outputs/excel/frequency_model_review.xlsx
+++ b/outputs/excel/frequency_model_review.xlsx
@@ -448,7 +448,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>predicted_claims</t>
+          <t>expected_claims</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -458,7 +458,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>predicted_frequency</t>
+          <t>expected_frequency</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -537,7 +537,7 @@
         <v>234</v>
       </c>
       <c r="F3" t="n">
-        <v>229.155168</v>
+        <v>229.16</v>
       </c>
       <c r="G3" t="n">
         <v>0.08563</v>
@@ -615,7 +615,7 @@
         <v>234</v>
       </c>
       <c r="F5" t="n">
-        <v>233.553935</v>
+        <v>233.55</v>
       </c>
       <c r="G5" t="n">
         <v>0.08563</v>
@@ -706,37 +706,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-2.717984</v>
+        <v>-3.481204</v>
       </c>
       <c r="C2" t="n">
-        <v>0.154613</v>
+        <v>0.127408</v>
       </c>
       <c r="D2" t="n">
-        <v>-17.579308</v>
+        <v>-27.323304</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>-3.021019</v>
+        <v>-3.730918</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.414949</v>
+        <v>-3.231489</v>
       </c>
       <c r="H2" t="n">
-        <v>0.066008</v>
+        <v>0.03077</v>
       </c>
       <c r="I2" t="n">
-        <v>0.048752</v>
+        <v>0.023971</v>
       </c>
       <c r="J2" t="n">
-        <v>0.08937199999999999</v>
+        <v>0.039499</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C(territory)[T.Suburban]</t>
+          <t>C(territory, Treatment(reference="Rural"))[T.Suburban]</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -770,7 +770,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C(territory)[T.Urban A]</t>
+          <t>C(territory, Treatment(reference="Rural"))[T.Urban A]</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -804,7 +804,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C(territory)[T.Urban B]</t>
+          <t>C(territory, Treatment(reference="Rural"))[T.Urban B]</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -838,307 +838,307 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C(driver_age_band)[T.25-39]</t>
+          <t>C(driver_age_band, Treatment(reference="40-64"))[T.16-24]</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.682046</v>
+        <v>0.882962</v>
       </c>
       <c r="C6" t="n">
-        <v>0.108299</v>
+        <v>0.100827</v>
       </c>
       <c r="D6" t="n">
-        <v>-6.297785</v>
+        <v>8.757223</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.894309</v>
+        <v>0.685346</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.469783</v>
+        <v>1.080579</v>
       </c>
       <c r="H6" t="n">
-        <v>0.5055809999999999</v>
+        <v>2.418052</v>
       </c>
       <c r="I6" t="n">
-        <v>0.40889</v>
+        <v>1.984458</v>
       </c>
       <c r="J6" t="n">
-        <v>0.625138</v>
+        <v>2.946386</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C(driver_age_band)[T.40-64]</t>
+          <t>C(driver_age_band, Treatment(reference="40-64"))[T.25-39]</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.882962</v>
+        <v>0.200916</v>
       </c>
       <c r="C7" t="n">
-        <v>0.100827</v>
+        <v>0.083341</v>
       </c>
       <c r="D7" t="n">
-        <v>-8.757223</v>
+        <v>2.410787</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>0.015918</v>
       </c>
       <c r="F7" t="n">
-        <v>-1.080579</v>
+        <v>0.037572</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.685346</v>
+        <v>0.364261</v>
       </c>
       <c r="H7" t="n">
-        <v>0.413556</v>
+        <v>1.222522</v>
       </c>
       <c r="I7" t="n">
-        <v>0.339399</v>
+        <v>1.038287</v>
       </c>
       <c r="J7" t="n">
-        <v>0.503916</v>
+        <v>1.43945</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C(driver_age_band)[T.65+]</t>
+          <t>C(driver_age_band, Treatment(reference="40-64"))[T.65+]</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.393056</v>
+        <v>0.489906</v>
       </c>
       <c r="C8" t="n">
-        <v>0.113757</v>
+        <v>0.090306</v>
       </c>
       <c r="D8" t="n">
-        <v>-3.45524</v>
+        <v>5.42495</v>
       </c>
       <c r="E8" t="n">
-        <v>0.00055</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.616015</v>
+        <v>0.31291</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.170097</v>
+        <v>0.666903</v>
       </c>
       <c r="H8" t="n">
-        <v>0.674991</v>
+        <v>1.632163</v>
       </c>
       <c r="I8" t="n">
-        <v>0.540093</v>
+        <v>1.367398</v>
       </c>
       <c r="J8" t="n">
-        <v>0.843583</v>
+        <v>1.948195</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C(vehicle_age_band)[T.13+]</t>
+          <t>C(vehicle_age_band, Treatment(reference="4-7"))[T.0-3]</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.515513</v>
+        <v>-0.163639</v>
       </c>
       <c r="C9" t="n">
-        <v>0.099032</v>
+        <v>0.106919</v>
       </c>
       <c r="D9" t="n">
-        <v>5.205518</v>
+        <v>-1.530491</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>0.125895</v>
       </c>
       <c r="F9" t="n">
-        <v>0.321414</v>
+        <v>-0.373197</v>
       </c>
       <c r="G9" t="n">
-        <v>0.709612</v>
+        <v>0.045919</v>
       </c>
       <c r="H9" t="n">
-        <v>1.674497</v>
+        <v>0.849048</v>
       </c>
       <c r="I9" t="n">
-        <v>1.379076</v>
+        <v>0.6885289999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>2.033203</v>
+        <v>1.04699</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C(vehicle_age_band)[T.4-7]</t>
+          <t>C(vehicle_age_band, Treatment(reference="4-7"))[T.13+]</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.163639</v>
+        <v>0.351874</v>
       </c>
       <c r="C10" t="n">
-        <v>0.106919</v>
+        <v>0.088896</v>
       </c>
       <c r="D10" t="n">
-        <v>1.530491</v>
+        <v>3.958284</v>
       </c>
       <c r="E10" t="n">
-        <v>0.125895</v>
+        <v>7.499999999999999e-05</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.045919</v>
+        <v>0.177642</v>
       </c>
       <c r="G10" t="n">
-        <v>0.373197</v>
+        <v>0.526106</v>
       </c>
       <c r="H10" t="n">
-        <v>1.177789</v>
+        <v>1.421729</v>
       </c>
       <c r="I10" t="n">
-        <v>0.9551190000000001</v>
+        <v>1.194397</v>
       </c>
       <c r="J10" t="n">
-        <v>1.452371</v>
+        <v>1.692329</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C(vehicle_age_band)[T.8-12]</t>
+          <t>C(vehicle_age_band, Treatment(reference="4-7"))[T.8-12]</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.321744</v>
+        <v>0.158104</v>
       </c>
       <c r="C11" t="n">
-        <v>0.103717</v>
+        <v>0.094108</v>
       </c>
       <c r="D11" t="n">
-        <v>3.10212</v>
+        <v>1.680026</v>
       </c>
       <c r="E11" t="n">
-        <v>0.001921</v>
+        <v>0.09295200000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>0.118461</v>
+        <v>-0.026345</v>
       </c>
       <c r="G11" t="n">
-        <v>0.525026</v>
+        <v>0.342553</v>
       </c>
       <c r="H11" t="n">
-        <v>1.379531</v>
+        <v>1.171289</v>
       </c>
       <c r="I11" t="n">
-        <v>1.125763</v>
+        <v>0.9739989999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>1.690503</v>
+        <v>1.40854</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C(vehicle_type)[T.Sedan]</t>
+          <t>C(vehicle_type, Treatment(reference="Sedan"))[T.SUV]</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.043896</v>
+        <v>0.043896</v>
       </c>
       <c r="C12" t="n">
         <v>0.077651</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.565303</v>
+        <v>0.565303</v>
       </c>
       <c r="E12" t="n">
         <v>0.571868</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.19609</v>
+        <v>-0.108297</v>
       </c>
       <c r="G12" t="n">
-        <v>0.108297</v>
+        <v>0.19609</v>
       </c>
       <c r="H12" t="n">
-        <v>0.957053</v>
+        <v>1.044874</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8219379999999999</v>
+        <v>0.897361</v>
       </c>
       <c r="J12" t="n">
-        <v>1.114379</v>
+        <v>1.216636</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C(vehicle_type)[T.Sports]</t>
+          <t>C(vehicle_type, Treatment(reference="Sedan"))[T.Sports]</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.672837</v>
+        <v>0.716734</v>
       </c>
       <c r="C13" t="n">
-        <v>0.125511</v>
+        <v>0.121276</v>
       </c>
       <c r="D13" t="n">
-        <v>5.360782</v>
+        <v>5.909925</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0.42684</v>
+        <v>0.479037</v>
       </c>
       <c r="G13" t="n">
-        <v>0.918834</v>
+        <v>0.954431</v>
       </c>
       <c r="H13" t="n">
-        <v>1.95979</v>
+        <v>2.047734</v>
       </c>
       <c r="I13" t="n">
-        <v>1.532408</v>
+        <v>1.614518</v>
       </c>
       <c r="J13" t="n">
-        <v>2.506367</v>
+        <v>2.597192</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C(vehicle_type)[T.Truck]</t>
+          <t>C(vehicle_type, Treatment(reference="Sedan"))[T.Truck]</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.199727</v>
+        <v>0.243623</v>
       </c>
       <c r="C14" t="n">
-        <v>0.099343</v>
+        <v>0.09396599999999999</v>
       </c>
       <c r="D14" t="n">
-        <v>2.010477</v>
+        <v>2.592679</v>
       </c>
       <c r="E14" t="n">
-        <v>0.044381</v>
+        <v>0.009523</v>
       </c>
       <c r="F14" t="n">
-        <v>0.005018</v>
+        <v>0.059454</v>
       </c>
       <c r="G14" t="n">
-        <v>0.394436</v>
+        <v>0.427793</v>
       </c>
       <c r="H14" t="n">
-        <v>1.221069</v>
+        <v>1.275864</v>
       </c>
       <c r="I14" t="n">
-        <v>1.005031</v>
+        <v>1.061257</v>
       </c>
       <c r="J14" t="n">
-        <v>1.483547</v>
+        <v>1.533869</v>
       </c>
     </row>
   </sheetData>

</xml_diff>